<commit_message>
Fix Empresa/Área mix-up in ATS/RPS generated formats
The Excel's "ÁREA" column actually identifies the worker's real
employer (a sister company/subsidiary within the group), not an
internal department — a single upload can span workers from several
legal entities. The generated formats were putting that value under
"Área:" while always stamping the one company name captured in
"Datos del centro de trabajo" under "Empresa:", which is wrong when
workers belong to different entities.

Now "Empresa:" is filled per worker from that column, and "Área:" is
left blank (no department data exists) for manual fill-in. Updated
the in-app help text and the two example templates' instructions to
explain this explicitly. generarFormatoAtsVerificacion and
generarFormatoEntrevistaRps no longer take the global company data
param, since it's unused now.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/plantilla-resultados-ats.xlsx
+++ b/public/plantillas/plantilla-resultados-ats.xlsx
@@ -401,7 +401,7 @@
   <dimension ref="A1:D3"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
     <col min="4" max="4" width="45.83203125" customWidth="1"/>
   </cols>
@@ -425,7 +425,7 @@
         <v>Juan Pérez López</v>
       </c>
       <c r="B2" t="str">
-        <v>Producción</v>
+        <v>Empresa Filial 1</v>
       </c>
       <c r="C2" t="str">
         <v>Si</v>
@@ -439,7 +439,7 @@
         <v>María González Ruiz</v>
       </c>
       <c r="B3" t="str">
-        <v>Administración</v>
+        <v>Empresa Filial 2</v>
       </c>
       <c r="C3" t="str">
         <v>No</v>
@@ -457,9 +457,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <cols>
-    <col min="1" max="1" width="90.83203125" customWidth="1"/>
+    <col min="1" max="1" width="100.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,27 +484,32 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>- La columna "¿REQUIERE ATENCIÓN CLÍNICA?" debe decir exactamente "Si" o "No".</v>
+        <v>- "ÁREA" debe traer la empresa o razón social real a la que pertenece el trabajador (por ejemplo, si el grupo tiene varias subsidiarias, va el nombre de la subsidiaria). Ese valor se usa como "Empresa:" en el formato generado; el campo "Área:" del formato queda en blanco para llenarse a mano.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>- Solo se genera el formato de verificación y la carta de canalización para quienes tengan "Si".</v>
+        <v>- La columna "¿REQUIERE ATENCIÓN CLÍNICA?" debe decir exactamente "Si" o "No".</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>- "MOTIVOS" es opcional: si se llena, aparece en el formato de verificación.</v>
+        <v>- Solo se genera el formato de verificación y la carta de canalización para quienes tengan "Si".</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>- "MOTIVOS" es opcional: si se llena, aparece en el formato de verificación.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>- Borra las filas de ejemplo antes de subir tu archivo real.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>